<commit_message>
Regenerate songlist.xlsx from data/songs.json (1911 songs)
The xlsx had not been refreshed since the 0.7.10 release while
data/songs.json (which the bot actually reads) advanced through 0.7.10,
0.8.0, and the Happy Meals codename. This re-syncs the xlsx with the
catalog the bot is serving.

Add scripts/regenerate-songlist-xlsx.js so this can be re-run any time
the JSON catalog changes ahead of a release. The script unzips the
existing xlsx, swaps in a freshly generated sheet1.xml built from
songs.json (preserving sheet name + column order: Title, Artist, Year,
Game, Original Game, Region, Release Date, Mode, Difficulty, Effort),
and re-zips. No new npm deps.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/songlist.xlsx
+++ b/songlist.xlsx
@@ -9,19 +9,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J1912"/>
-  <cols>
-    <col min="1" max="1" width="34" customWidth="1"/>
-    <col min="2" max="2" width="30" customWidth="1"/>
-    <col min="3" max="3" width="10" customWidth="1"/>
-    <col min="4" max="4" width="24" customWidth="1"/>
-    <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="18" customWidth="1"/>
-    <col min="7" max="7" width="20" customWidth="1"/>
-    <col min="8" max="8" width="16" customWidth="1"/>
-    <col min="9" max="9" width="16" customWidth="1"/>
-    <col min="10" max="10" width="16" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -42688,7 +42675,7 @@
       </c>
       <c r="C854" t="inlineStr">
         <is>
-          <t>None</t>
+          <t/>
         </is>
       </c>
       <c r="D854" t="inlineStr">
@@ -42740,7 +42727,7 @@
       </c>
       <c r="C855" t="inlineStr">
         <is>
-          <t>None</t>
+          <t/>
         </is>
       </c>
       <c r="D855" t="inlineStr">
@@ -42792,7 +42779,7 @@
       </c>
       <c r="C856" t="inlineStr">
         <is>
-          <t>None</t>
+          <t/>
         </is>
       </c>
       <c r="D856" t="inlineStr">
@@ -42844,7 +42831,7 @@
       </c>
       <c r="C857" t="inlineStr">
         <is>
-          <t>None</t>
+          <t/>
         </is>
       </c>
       <c r="D857" t="inlineStr">
@@ -42896,7 +42883,7 @@
       </c>
       <c r="C858" t="inlineStr">
         <is>
-          <t>None</t>
+          <t/>
         </is>
       </c>
       <c r="D858" t="inlineStr">
@@ -49798,7 +49785,7 @@
       </c>
       <c r="C996" t="inlineStr">
         <is>
-          <t>None</t>
+          <t/>
         </is>
       </c>
       <c r="D996" t="inlineStr">
@@ -96200,6 +96187,5 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J1912"/>
 </worksheet>
 </file>
</xml_diff>